<commit_message>
Ajustar inventario mobile e cache operacional
</commit_message>
<xml_diff>
--- a/estoque_app/dados_exemplo.xlsx
+++ b/estoque_app/dados_exemplo.xlsx
@@ -423,15 +423,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,22 +448,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>SALDO_ATUAL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ESTOQUE_MINIMO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>UNIDADE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>CATEGORIA</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>LOCALIZACAO</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>ESTOQUE_MINIMO</t>
         </is>
       </c>
     </row>
@@ -477,23 +483,26 @@
           <t>Parafuso sextavado M8 x 30 zincado</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="n">
+        <v>125</v>
+      </c>
+      <c r="D2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>UN</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Fixadores</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>A1-01</t>
         </is>
-      </c>
-      <c r="F2" t="n">
-        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -507,23 +516,24 @@
           <t>Cabo eletrico flexivel 2,5 mm preto</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="n">
+        <v>80</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Eletrica</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>B2-04</t>
         </is>
-      </c>
-      <c r="F3" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -537,23 +547,26 @@
           <t>Conector pneumatico reto 1/4</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>UN</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Pneumatica</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>C3-02</t>
         </is>
-      </c>
-      <c r="F4" t="n">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizar estoque, empenhos e fila local
</commit_message>
<xml_diff>
--- a/estoque_app/dados_exemplo.xlsx
+++ b/estoque_app/dados_exemplo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SKUs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKUs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Substituir nomenclatura SKU por COD
</commit_message>
<xml_diff>
--- a/estoque_app/dados_exemplo.xlsx
+++ b/estoque_app/dados_exemplo.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKUs" sheetId="1" r:id="R261fa3d6fd5845a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codigos" sheetId="1" r:id="R59ac3567bb26453e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -368,7 +368,7 @@
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>SKU</x:v>
+        <x:v>COD</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
         <x:v>DESCRICAO</x:v>
@@ -455,6 +455,7 @@
       <x:c r="D5" s="4"/>
       <x:c r="E5" s="4"/>
       <x:c r="F5" s="6"/>
+      <x:c r="G5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="5"/>
@@ -463,6 +464,7 @@
       <x:c r="D6" s="4"/>
       <x:c r="E6" s="4"/>
       <x:c r="F6" s="6"/>
+      <x:c r="G6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5"/>
@@ -471,6 +473,7 @@
       <x:c r="D7" s="4"/>
       <x:c r="E7" s="4"/>
       <x:c r="F7" s="6"/>
+      <x:c r="G7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5"/>
@@ -479,6 +482,7 @@
       <x:c r="D8" s="4"/>
       <x:c r="E8" s="4"/>
       <x:c r="F8" s="6"/>
+      <x:c r="G8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="5"/>
@@ -487,6 +491,7 @@
       <x:c r="D9" s="4"/>
       <x:c r="E9" s="4"/>
       <x:c r="F9" s="6"/>
+      <x:c r="G9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5"/>
@@ -495,6 +500,7 @@
       <x:c r="D10" s="4"/>
       <x:c r="E10" s="4"/>
       <x:c r="F10" s="6"/>
+      <x:c r="G10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="5"/>
@@ -503,6 +509,7 @@
       <x:c r="D11" s="4"/>
       <x:c r="E11" s="4"/>
       <x:c r="F11" s="6"/>
+      <x:c r="G11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="5"/>
@@ -511,6 +518,7 @@
       <x:c r="D12" s="4"/>
       <x:c r="E12" s="4"/>
       <x:c r="F12" s="6"/>
+      <x:c r="G12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="5"/>
@@ -519,6 +527,7 @@
       <x:c r="D13" s="4"/>
       <x:c r="E13" s="4"/>
       <x:c r="F13" s="6"/>
+      <x:c r="G13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="5"/>
@@ -527,6 +536,7 @@
       <x:c r="D14" s="4"/>
       <x:c r="E14" s="4"/>
       <x:c r="F14" s="6"/>
+      <x:c r="G14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="5"/>
@@ -535,6 +545,7 @@
       <x:c r="D15" s="4"/>
       <x:c r="E15" s="4"/>
       <x:c r="F15" s="6"/>
+      <x:c r="G15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="5"/>
@@ -543,6 +554,7 @@
       <x:c r="D16" s="4"/>
       <x:c r="E16" s="4"/>
       <x:c r="F16" s="6"/>
+      <x:c r="G16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5"/>
@@ -551,6 +563,7 @@
       <x:c r="D17" s="4"/>
       <x:c r="E17" s="4"/>
       <x:c r="F17" s="6"/>
+      <x:c r="G17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="5"/>
@@ -559,6 +572,7 @@
       <x:c r="D18" s="4"/>
       <x:c r="E18" s="4"/>
       <x:c r="F18" s="6"/>
+      <x:c r="G18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="5"/>
@@ -567,6 +581,7 @@
       <x:c r="D19" s="4"/>
       <x:c r="E19" s="4"/>
       <x:c r="F19" s="6"/>
+      <x:c r="G19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="5"/>
@@ -575,6 +590,7 @@
       <x:c r="D20" s="4"/>
       <x:c r="E20" s="4"/>
       <x:c r="F20" s="6"/>
+      <x:c r="G20"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>